<commit_message>
Save local automation changes
</commit_message>
<xml_diff>
--- a/Localisation/suite_GFL_Croatia/tst_GEM-LOC-CROATIA-PeakPower-SoftTissueCharacters/testdata/Peakpower.xlsx
+++ b/Localisation/suite_GFL_Croatia/tst_GEM-LOC-CROATIA-PeakPower-SoftTissueCharacters/testdata/Peakpower.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Jaka</t>
   </si>
   <si>
-    <t xml:space="preserve">Srednji</t>
+    <t xml:space="preserve">SREDNJA</t>
   </si>
   <si>
     <t xml:space="preserve">Slaba</t>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">POSTUPAK</t>
   </si>
   <si>
-    <t xml:space="preserve">Incision</t>
+    <t xml:space="preserve">REZ</t>
   </si>
   <si>
     <t xml:space="preserve">UREDI</t>
@@ -62,7 +62,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -91,6 +91,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -102,7 +109,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -110,6 +117,13 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -136,7 +150,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -150,6 +164,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -204,7 +222,7 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -238,11 +256,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="4" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>